<commit_message>
Procurement Reference v2.1: Quotations only under £100k (new V0 level), Project types column (Remeasurement on External works only), TN4 for negotiated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Projento_Procurement_Reference.xlsx
+++ b/Projento_Procurement_Reference.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\estates-ai-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E2749D-BB65-4121-8491-FF50B8FC0451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0250CFB5-F4BC-484F-B409-DCBDCE876166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Read Me" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,9 @@
     <sheet name="4. Check" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. Options'!$A$1:$Y$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. Options'!$A$1:$Z$16</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr fullCalcOnLoad="1" calcId="191029"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -37,7 +37,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="D27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="D28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="312">
   <si>
     <t>Projento — Procurement Reference v2</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0 · 28 September 2026 · Nabil Kayali · replaces v1</t>
-  </si>
-  <si>
     <t>Purpose</t>
   </si>
   <si>
@@ -975,6 +972,24 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>V0</t>
+  </si>
+  <si>
+    <t>V0 Under £100k</t>
+  </si>
+  <si>
+    <t>Project types</t>
+  </si>
+  <si>
+    <t>External works only</t>
+  </si>
+  <si>
+    <t>2.1 · 10 October 2026 · Nabil Kayali · replaces v2.0 (value level V0 under £100k; Quotations only under £100k; Project types column — Remeasurement for External works only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JCT — V0/V1 under £1m</t>
   </si>
 </sst>
 </file>
@@ -1157,7 +1172,57 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFBFBFBF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8D7D3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD5E8D4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFBFBFBF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8D7D3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD5E8D4"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1456,20 +1521,20 @@
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>2</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1478,40 +1543,40 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1520,40 +1585,40 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" s="2"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -1562,72 +1627,72 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B17" s="2"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -1636,10 +1701,10 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -1648,40 +1713,40 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B29" s="2"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -1690,40 +1755,40 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B35" s="2"/>
     </row>
     <row r="36" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1734,7 +1799,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1747,368 +1812,379 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="D2" s="8">
+        <v>0</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D3" s="8">
+        <v>100000</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="8">
-        <v>0</v>
-      </c>
-      <c r="E2" s="7" t="s">
+      <c r="F3" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="F2" s="7" t="s">
+    </row>
+    <row r="4" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D4" s="11">
+        <v>1000000</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="11">
-        <v>1000000</v>
-      </c>
-      <c r="E3" s="10" t="s">
+      <c r="C5" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="12">
+        <f>$D$29</f>
+        <v>4327500</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="7" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="12">
-        <f>$D$28</f>
-        <v>4327500</v>
-      </c>
-      <c r="E4" s="7" t="s">
+      <c r="C6" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="11">
+        <v>20000000</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="10" t="s">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="D5" s="11">
-        <v>20000000</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D7" s="13">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="D6" s="13">
-        <v>0</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="F7" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="7" t="s">
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="10" t="s">
+      <c r="C8" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="D8" s="14">
+        <v>27</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D7" s="14">
-        <v>27</v>
-      </c>
-      <c r="E7" s="10" t="s">
+      <c r="C9" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" s="13">
+        <v>53</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="C8" s="7" t="s">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="D8" s="13">
-        <v>53</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="10" t="s">
+      <c r="C10" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="D10" s="14">
+        <v>0</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="D9" s="14">
-        <v>0</v>
-      </c>
-      <c r="E9" s="10" t="s">
+      <c r="F10" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F9" s="10" t="s">
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="7" t="s">
+      <c r="C11" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D11" s="13">
+        <v>2</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D10" s="13">
-        <v>2</v>
-      </c>
-      <c r="E10" s="7" t="s">
+      <c r="F11" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="F10" s="7" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="10" t="s">
+      <c r="C12" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="D12" s="14">
+        <v>4</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="D11" s="14">
-        <v>4</v>
-      </c>
-      <c r="E11" s="10" t="s">
+      <c r="F12" s="10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="7" t="s">
+      <c r="C13" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D13" s="7"/>
+      <c r="E13" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7" t="s">
+      <c r="F13" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="F12" s="7" t="s">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="10" t="s">
+      <c r="C14" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="D14" s="10"/>
+      <c r="E14" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10" t="s">
+      <c r="F14" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="7" t="s">
+      <c r="C15" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D15" s="7"/>
+      <c r="E15" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7" t="s">
+      <c r="F15" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="10" t="s">
+      <c r="C16" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="D16" s="10"/>
+      <c r="E16" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10" t="s">
+      <c r="F16" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D17" s="7"/>
+      <c r="E17" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7" t="s">
+      <c r="F17" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B17" s="10" t="s">
+      <c r="C18" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="D18" s="10"/>
+      <c r="E18" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10" t="s">
+      <c r="F18" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B18" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D19" s="7"/>
+      <c r="E19" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7" t="s">
+      <c r="F19" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="D21" s="17">
-        <v>1</v>
-      </c>
-      <c r="E21" s="18"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D22" s="17">
         <v>1</v>
@@ -2117,7 +2193,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D23" s="17">
         <v>1</v>
@@ -2126,41 +2202,50 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="D24" s="17">
+        <v>1</v>
+      </c>
+      <c r="E24" s="18"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="D25" s="17">
+        <v>2</v>
+      </c>
+      <c r="E25" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="D24" s="17">
-        <v>2</v>
-      </c>
-      <c r="E24" s="18" t="s">
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="15" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="D27" s="19">
-        <v>5193000</v>
-      </c>
-      <c r="E27" s="18" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="D28" s="19">
+        <v>5193000</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="D29" s="20">
+        <f>D28/1.2</f>
+        <v>4327500</v>
+      </c>
+      <c r="E29" s="18" t="s">
         <v>125</v>
-      </c>
-      <c r="D28" s="20">
-        <f>D27/1.2</f>
-        <v>4327500</v>
-      </c>
-      <c r="E28" s="18" t="s">
-        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -2172,7 +2257,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Y18"/>
+  <dimension ref="A1:AA18"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -2183,190 +2268,200 @@
     <col min="6" max="6" width="46" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="24" width="10" customWidth="1"/>
-    <col min="25" max="25" width="16" customWidth="1"/>
+    <col min="9" max="25" width="10" customWidth="1"/>
+    <col min="26" max="27" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="R1" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z1" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="T1" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="U1" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="V1" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="W1" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="X1" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="Y1" s="5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="B2" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="7" t="s">
         <v>138</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>139</v>
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="I2" s="21">
+        <v>2</v>
+      </c>
+      <c r="J2" s="21">
+        <v>2</v>
+      </c>
+      <c r="K2" s="21">
+        <v>2</v>
+      </c>
+      <c r="L2" s="21">
+        <v>1</v>
+      </c>
+      <c r="M2" s="21">
+        <v>1</v>
+      </c>
+      <c r="N2" s="21">
+        <v>2</v>
+      </c>
+      <c r="O2" s="21">
+        <v>2</v>
+      </c>
+      <c r="P2" s="21">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="21">
+        <v>2</v>
+      </c>
+      <c r="R2" s="21">
+        <v>1</v>
+      </c>
+      <c r="S2" s="21">
+        <v>0</v>
+      </c>
+      <c r="T2" s="21">
+        <v>2</v>
+      </c>
+      <c r="U2" s="21">
+        <v>2</v>
+      </c>
+      <c r="V2" s="21">
+        <v>0</v>
+      </c>
+      <c r="W2" s="21">
+        <v>2</v>
+      </c>
+      <c r="X2" s="21">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="21">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="21">
+        <v>2</v>
+      </c>
+      <c r="AA2" s="21"/>
+    </row>
+    <row r="3" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="I2" s="21">
-        <v>2</v>
-      </c>
-      <c r="J2" s="21">
-        <v>2</v>
-      </c>
-      <c r="K2" s="21">
-        <v>1</v>
-      </c>
-      <c r="L2" s="21">
-        <v>1</v>
-      </c>
-      <c r="M2" s="21">
-        <v>2</v>
-      </c>
-      <c r="N2" s="21">
-        <v>2</v>
-      </c>
-      <c r="O2" s="21">
-        <v>1</v>
-      </c>
-      <c r="P2" s="21">
-        <v>2</v>
-      </c>
-      <c r="Q2" s="21">
-        <v>1</v>
-      </c>
-      <c r="R2" s="21">
-        <v>0</v>
-      </c>
-      <c r="S2" s="21">
-        <v>2</v>
-      </c>
-      <c r="T2" s="21">
-        <v>2</v>
-      </c>
-      <c r="U2" s="21">
-        <v>0</v>
-      </c>
-      <c r="V2" s="21">
-        <v>2</v>
-      </c>
-      <c r="W2" s="21">
-        <v>1</v>
-      </c>
-      <c r="X2" s="21">
-        <v>1</v>
-      </c>
-      <c r="Y2" s="21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="B3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>145</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I3" s="21">
         <v>1</v>
       </c>
       <c r="J3" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" s="21">
         <v>2</v>
@@ -2375,10 +2470,10 @@
         <v>2</v>
       </c>
       <c r="M3" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N3" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O3" s="21">
         <v>2</v>
@@ -2387,7 +2482,7 @@
         <v>2</v>
       </c>
       <c r="Q3" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R3" s="21">
         <v>1</v>
@@ -2396,695 +2491,733 @@
         <v>1</v>
       </c>
       <c r="T3" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U3" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V3" s="21">
         <v>1</v>
       </c>
       <c r="W3" s="21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X3" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="21">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:25" ht="51" x14ac:dyDescent="0.25">
+      <c r="Z3" s="21">
+        <v>1</v>
+      </c>
+      <c r="AA3" s="21"/>
+    </row>
+    <row r="4" spans="1:27" ht="51" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>150</v>
       </c>
       <c r="G4" s="7"/>
       <c r="H4" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I4" s="21">
         <v>0</v>
       </c>
       <c r="J4" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L4" s="21">
         <v>2</v>
       </c>
       <c r="M4" s="21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N4" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P4" s="21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q4" s="21">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R4" s="21">
         <v>2</v>
       </c>
       <c r="S4" s="21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T4" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U4" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V4" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W4" s="21">
         <v>1</v>
       </c>
       <c r="X4" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y4" s="21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="Z4" s="21">
+        <v>1</v>
+      </c>
+      <c r="AA4" s="21"/>
+    </row>
+    <row r="5" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="E5" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="F5" s="10" t="s">
         <v>154</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>155</v>
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I5" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="J5" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="K5" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="L5" s="21">
+        <v>0</v>
+      </c>
+      <c r="M5" s="21">
+        <v>2</v>
+      </c>
+      <c r="N5" s="21">
+        <v>0</v>
+      </c>
+      <c r="O5" s="21">
+        <v>1</v>
+      </c>
+      <c r="P5" s="21">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="21">
+        <v>0</v>
+      </c>
+      <c r="R5" s="21">
+        <v>1</v>
+      </c>
+      <c r="S5" s="21">
+        <v>2</v>
+      </c>
+      <c r="T5" s="21">
+        <v>0</v>
+      </c>
+      <c r="U5" s="21">
+        <v>0</v>
+      </c>
+      <c r="V5" s="21">
+        <v>2</v>
+      </c>
+      <c r="W5" s="21">
+        <v>2</v>
+      </c>
+      <c r="X5" s="21">
+        <v>2</v>
+      </c>
+      <c r="Y5" s="21">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="21">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="21"/>
+    </row>
+    <row r="6" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="J5" s="21" t="s">
-        <v>156</v>
-      </c>
-      <c r="K5" s="21">
-        <v>0</v>
-      </c>
-      <c r="L5" s="21">
-        <v>2</v>
-      </c>
-      <c r="M5" s="21">
-        <v>0</v>
-      </c>
-      <c r="N5" s="21">
-        <v>1</v>
-      </c>
-      <c r="O5" s="21">
-        <v>2</v>
-      </c>
-      <c r="P5" s="21">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="21">
-        <v>1</v>
-      </c>
-      <c r="R5" s="21">
-        <v>2</v>
-      </c>
-      <c r="S5" s="21">
-        <v>0</v>
-      </c>
-      <c r="T5" s="21">
-        <v>0</v>
-      </c>
-      <c r="U5" s="21">
-        <v>2</v>
-      </c>
-      <c r="V5" s="21">
-        <v>2</v>
-      </c>
-      <c r="W5" s="21">
-        <v>2</v>
-      </c>
-      <c r="X5" s="21">
-        <v>1</v>
-      </c>
-      <c r="Y5" s="21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="B6" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="I6" s="21">
+        <v>2</v>
+      </c>
+      <c r="J6" s="21">
+        <v>2</v>
+      </c>
+      <c r="K6" s="21">
+        <v>2</v>
+      </c>
+      <c r="L6" s="21">
+        <v>2</v>
+      </c>
+      <c r="M6" s="21">
+        <v>1</v>
+      </c>
+      <c r="N6" s="21">
+        <v>2</v>
+      </c>
+      <c r="O6" s="21">
+        <v>2</v>
+      </c>
+      <c r="P6" s="21">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="21">
+        <v>2</v>
+      </c>
+      <c r="R6" s="21">
+        <v>1</v>
+      </c>
+      <c r="S6" s="21">
+        <v>0</v>
+      </c>
+      <c r="T6" s="21">
+        <v>2</v>
+      </c>
+      <c r="U6" s="21">
+        <v>2</v>
+      </c>
+      <c r="V6" s="21">
+        <v>1</v>
+      </c>
+      <c r="W6" s="21">
+        <v>1</v>
+      </c>
+      <c r="X6" s="21">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="21">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="21">
+        <v>2</v>
+      </c>
+      <c r="AA6" s="21"/>
+    </row>
+    <row r="7" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="I6" s="21">
-        <v>2</v>
-      </c>
-      <c r="J6" s="21">
-        <v>2</v>
-      </c>
-      <c r="K6" s="21">
-        <v>2</v>
-      </c>
-      <c r="L6" s="21">
-        <v>1</v>
-      </c>
-      <c r="M6" s="21">
-        <v>2</v>
-      </c>
-      <c r="N6" s="21">
-        <v>2</v>
-      </c>
-      <c r="O6" s="21">
-        <v>1</v>
-      </c>
-      <c r="P6" s="21">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="21">
-        <v>1</v>
-      </c>
-      <c r="R6" s="21">
-        <v>0</v>
-      </c>
-      <c r="S6" s="21">
-        <v>2</v>
-      </c>
-      <c r="T6" s="21">
-        <v>2</v>
-      </c>
-      <c r="U6" s="21">
-        <v>1</v>
-      </c>
-      <c r="V6" s="21">
-        <v>1</v>
-      </c>
-      <c r="W6" s="21">
-        <v>0</v>
-      </c>
-      <c r="X6" s="21">
-        <v>1</v>
-      </c>
-      <c r="Y6" s="21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="B7" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="E7" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="F7" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="H7" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="I7" s="21">
+        <v>0</v>
+      </c>
+      <c r="J7" s="21">
+        <v>0</v>
+      </c>
+      <c r="K7" s="21">
+        <v>1</v>
+      </c>
+      <c r="L7" s="21">
+        <v>2</v>
+      </c>
+      <c r="M7" s="21">
+        <v>2</v>
+      </c>
+      <c r="N7" s="21">
+        <v>0</v>
+      </c>
+      <c r="O7" s="21">
+        <v>1</v>
+      </c>
+      <c r="P7" s="21">
+        <v>2</v>
+      </c>
+      <c r="Q7" s="21">
+        <v>0</v>
+      </c>
+      <c r="R7" s="21">
+        <v>2</v>
+      </c>
+      <c r="S7" s="21">
+        <v>1</v>
+      </c>
+      <c r="T7" s="21">
+        <v>0</v>
+      </c>
+      <c r="U7" s="21">
+        <v>2</v>
+      </c>
+      <c r="V7" s="21">
+        <v>1</v>
+      </c>
+      <c r="W7" s="21">
+        <v>0</v>
+      </c>
+      <c r="X7" s="21">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="21">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="21">
+        <v>1</v>
+      </c>
+      <c r="AA7" s="21"/>
+    </row>
+    <row r="8" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="H7" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="I7" s="21">
-        <v>0</v>
-      </c>
-      <c r="J7" s="21">
-        <v>1</v>
-      </c>
-      <c r="K7" s="21">
-        <v>2</v>
-      </c>
-      <c r="L7" s="21">
-        <v>2</v>
-      </c>
-      <c r="M7" s="21">
-        <v>0</v>
-      </c>
-      <c r="N7" s="21">
-        <v>1</v>
-      </c>
-      <c r="O7" s="21">
-        <v>2</v>
-      </c>
-      <c r="P7" s="21">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="21">
-        <v>2</v>
-      </c>
-      <c r="R7" s="21">
-        <v>1</v>
-      </c>
-      <c r="S7" s="21">
-        <v>0</v>
-      </c>
-      <c r="T7" s="21">
-        <v>2</v>
-      </c>
-      <c r="U7" s="21">
-        <v>1</v>
-      </c>
-      <c r="V7" s="21">
-        <v>0</v>
-      </c>
-      <c r="W7" s="21">
-        <v>1</v>
-      </c>
-      <c r="X7" s="21">
-        <v>1</v>
-      </c>
-      <c r="Y7" s="21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="B8" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="F8" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="G8" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="I8" s="21">
+        <v>0</v>
+      </c>
+      <c r="J8" s="21">
+        <v>0</v>
+      </c>
+      <c r="K8" s="21">
+        <v>1</v>
+      </c>
+      <c r="L8" s="21">
+        <v>2</v>
+      </c>
+      <c r="M8" s="21">
+        <v>2</v>
+      </c>
+      <c r="N8" s="21">
+        <v>0</v>
+      </c>
+      <c r="O8" s="21">
+        <v>1</v>
+      </c>
+      <c r="P8" s="21">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="21">
+        <v>0</v>
+      </c>
+      <c r="R8" s="21">
+        <v>1</v>
+      </c>
+      <c r="S8" s="21">
+        <v>2</v>
+      </c>
+      <c r="T8" s="21">
+        <v>1</v>
+      </c>
+      <c r="U8" s="21">
+        <v>0</v>
+      </c>
+      <c r="V8" s="21">
+        <v>2</v>
+      </c>
+      <c r="W8" s="21">
+        <v>1</v>
+      </c>
+      <c r="X8" s="21">
+        <v>2</v>
+      </c>
+      <c r="Y8" s="21">
+        <v>2</v>
+      </c>
+      <c r="Z8" s="21">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="21"/>
+    </row>
+    <row r="9" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="G8" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="I8" s="21">
-        <v>0</v>
-      </c>
-      <c r="J8" s="21">
-        <v>1</v>
-      </c>
-      <c r="K8" s="21">
-        <v>2</v>
-      </c>
-      <c r="L8" s="21">
-        <v>2</v>
-      </c>
-      <c r="M8" s="21">
-        <v>0</v>
-      </c>
-      <c r="N8" s="21">
-        <v>1</v>
-      </c>
-      <c r="O8" s="21">
-        <v>2</v>
-      </c>
-      <c r="P8" s="21">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="21">
-        <v>1</v>
-      </c>
-      <c r="R8" s="21">
-        <v>2</v>
-      </c>
-      <c r="S8" s="21">
-        <v>1</v>
-      </c>
-      <c r="T8" s="21">
-        <v>0</v>
-      </c>
-      <c r="U8" s="21">
-        <v>2</v>
-      </c>
-      <c r="V8" s="21">
-        <v>1</v>
-      </c>
-      <c r="W8" s="21">
-        <v>2</v>
-      </c>
-      <c r="X8" s="21">
-        <v>2</v>
-      </c>
-      <c r="Y8" s="21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="B9" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="E9" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="F9" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="G9" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="I9" s="21">
+        <v>2</v>
+      </c>
+      <c r="J9" s="21">
+        <v>2</v>
+      </c>
+      <c r="K9" s="21">
+        <v>2</v>
+      </c>
+      <c r="L9" s="21">
+        <v>1</v>
+      </c>
+      <c r="M9" s="21">
+        <v>1</v>
+      </c>
+      <c r="N9" s="21">
+        <v>1</v>
+      </c>
+      <c r="O9" s="21">
+        <v>2</v>
+      </c>
+      <c r="P9" s="21">
+        <v>2</v>
+      </c>
+      <c r="Q9" s="21">
+        <v>1</v>
+      </c>
+      <c r="R9" s="21">
+        <v>2</v>
+      </c>
+      <c r="S9" s="21">
+        <v>2</v>
+      </c>
+      <c r="T9" s="21">
+        <v>1</v>
+      </c>
+      <c r="U9" s="21">
+        <v>0</v>
+      </c>
+      <c r="V9" s="21">
+        <v>2</v>
+      </c>
+      <c r="W9" s="21">
+        <v>1</v>
+      </c>
+      <c r="X9" s="21">
+        <v>2</v>
+      </c>
+      <c r="Y9" s="21">
+        <v>1</v>
+      </c>
+      <c r="Z9" s="21">
+        <v>1</v>
+      </c>
+      <c r="AA9" s="21" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="G9" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="I9" s="21">
-        <v>2</v>
-      </c>
-      <c r="J9" s="21">
-        <v>2</v>
-      </c>
-      <c r="K9" s="21">
-        <v>1</v>
-      </c>
-      <c r="L9" s="21">
-        <v>1</v>
-      </c>
-      <c r="M9" s="21">
-        <v>1</v>
-      </c>
-      <c r="N9" s="21">
-        <v>2</v>
-      </c>
-      <c r="O9" s="21">
-        <v>2</v>
-      </c>
-      <c r="P9" s="21">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="21">
-        <v>2</v>
-      </c>
-      <c r="R9" s="21">
-        <v>2</v>
-      </c>
-      <c r="S9" s="21">
-        <v>1</v>
-      </c>
-      <c r="T9" s="21">
-        <v>0</v>
-      </c>
-      <c r="U9" s="21">
-        <v>2</v>
-      </c>
-      <c r="V9" s="21">
-        <v>1</v>
-      </c>
-      <c r="W9" s="21">
-        <v>2</v>
-      </c>
-      <c r="X9" s="21">
-        <v>1</v>
-      </c>
-      <c r="Y9" s="21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="B10" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="F10" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="H10" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="I10" s="21">
+        <v>1</v>
+      </c>
+      <c r="J10" s="21">
+        <v>1</v>
+      </c>
+      <c r="K10" s="21">
+        <v>0</v>
+      </c>
+      <c r="L10" s="21">
+        <v>0</v>
+      </c>
+      <c r="M10" s="21">
+        <v>1</v>
+      </c>
+      <c r="N10" s="21">
+        <v>2</v>
+      </c>
+      <c r="O10" s="21">
+        <v>1</v>
+      </c>
+      <c r="P10" s="21">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="21">
+        <v>0</v>
+      </c>
+      <c r="R10" s="21">
+        <v>1</v>
+      </c>
+      <c r="S10" s="21">
+        <v>2</v>
+      </c>
+      <c r="T10" s="21">
+        <v>0</v>
+      </c>
+      <c r="U10" s="21">
+        <v>0</v>
+      </c>
+      <c r="V10" s="21">
+        <v>2</v>
+      </c>
+      <c r="W10" s="21">
+        <v>1</v>
+      </c>
+      <c r="X10" s="21">
+        <v>2</v>
+      </c>
+      <c r="Y10" s="21">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="21">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="21"/>
+    </row>
+    <row r="11" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="H10" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="I10" s="21">
-        <v>1</v>
-      </c>
-      <c r="J10" s="21">
-        <v>0</v>
-      </c>
-      <c r="K10" s="21">
-        <v>0</v>
-      </c>
-      <c r="L10" s="21">
-        <v>1</v>
-      </c>
-      <c r="M10" s="21">
-        <v>2</v>
-      </c>
-      <c r="N10" s="21">
-        <v>1</v>
-      </c>
-      <c r="O10" s="21">
-        <v>1</v>
-      </c>
-      <c r="P10" s="21">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="21">
-        <v>1</v>
-      </c>
-      <c r="R10" s="21">
-        <v>2</v>
-      </c>
-      <c r="S10" s="21">
-        <v>0</v>
-      </c>
-      <c r="T10" s="21">
-        <v>0</v>
-      </c>
-      <c r="U10" s="21">
-        <v>2</v>
-      </c>
-      <c r="V10" s="21">
-        <v>1</v>
-      </c>
-      <c r="W10" s="21">
-        <v>2</v>
-      </c>
-      <c r="X10" s="21">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+      <c r="B11" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="E11" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="F11" s="10" t="s">
         <v>188</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>189</v>
       </c>
       <c r="G11" s="10"/>
       <c r="H11" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I11" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J11" s="21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K11" s="21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L11" s="21" t="s">
-        <v>156</v>
-      </c>
-      <c r="M11" s="21">
-        <v>2</v>
+        <v>155</v>
+      </c>
+      <c r="M11" s="21" t="s">
+        <v>155</v>
       </c>
       <c r="N11" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O11" s="21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P11" s="21">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R11" s="21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T11" s="21">
         <v>1</v>
       </c>
       <c r="U11" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V11" s="21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W11" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X11" s="21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y11" s="21">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="Z11" s="21">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="21"/>
+    </row>
+    <row r="12" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="6" t="s">
+      <c r="D12" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="E12" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="F12" s="7" t="s">
         <v>193</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>194</v>
       </c>
       <c r="G12" s="7"/>
       <c r="H12" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I12" s="21">
         <v>1</v>
       </c>
       <c r="J12" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" s="21">
         <v>2</v>
       </c>
       <c r="L12" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M12" s="21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N12" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O12" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P12" s="21">
         <v>2</v>
       </c>
       <c r="Q12" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" s="21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" s="21">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T12" s="21">
         <v>2</v>
       </c>
       <c r="U12" s="21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V12" s="21">
         <v>0</v>
@@ -3096,31 +3229,35 @@
         <v>0</v>
       </c>
       <c r="Y12" s="21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="21">
+        <v>2</v>
+      </c>
+      <c r="AA12" s="21"/>
+    </row>
+    <row r="13" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="E13" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="F13" s="10" t="s">
         <v>198</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>199</v>
       </c>
       <c r="G13" s="10"/>
       <c r="H13" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I13" s="21">
         <v>2</v>
@@ -3129,7 +3266,7 @@
         <v>2</v>
       </c>
       <c r="K13" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L13" s="21">
         <v>1</v>
@@ -3138,7 +3275,7 @@
         <v>1</v>
       </c>
       <c r="N13" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" s="21">
         <v>2</v>
@@ -3150,127 +3287,135 @@
         <v>2</v>
       </c>
       <c r="R13" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T13" s="21">
         <v>2</v>
       </c>
       <c r="U13" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V13" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W13" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X13" s="21">
         <v>1</v>
       </c>
       <c r="Y13" s="21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="Z13" s="21">
+        <v>2</v>
+      </c>
+      <c r="AA13" s="21"/>
+    </row>
+    <row r="14" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="6" t="s">
+      <c r="D14" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="F14" s="7" t="s">
         <v>203</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>204</v>
       </c>
       <c r="G14" s="7"/>
       <c r="H14" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="I14" s="21">
+        <v>1</v>
+      </c>
+      <c r="J14" s="21">
+        <v>1</v>
+      </c>
+      <c r="K14" s="21">
+        <v>2</v>
+      </c>
+      <c r="L14" s="21">
+        <v>2</v>
+      </c>
+      <c r="M14" s="21">
+        <v>2</v>
+      </c>
+      <c r="N14" s="21">
+        <v>1</v>
+      </c>
+      <c r="O14" s="21">
+        <v>2</v>
+      </c>
+      <c r="P14" s="21">
+        <v>2</v>
+      </c>
+      <c r="Q14" s="21">
+        <v>1</v>
+      </c>
+      <c r="R14" s="21">
+        <v>2</v>
+      </c>
+      <c r="S14" s="21">
+        <v>2</v>
+      </c>
+      <c r="T14" s="21">
+        <v>1</v>
+      </c>
+      <c r="U14" s="21">
+        <v>2</v>
+      </c>
+      <c r="V14" s="21">
+        <v>1</v>
+      </c>
+      <c r="W14" s="21">
+        <v>1</v>
+      </c>
+      <c r="X14" s="21">
+        <v>1</v>
+      </c>
+      <c r="Y14" s="21">
+        <v>1</v>
+      </c>
+      <c r="Z14" s="21">
+        <v>2</v>
+      </c>
+      <c r="AA14" s="21"/>
+    </row>
+    <row r="15" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="I14" s="21">
-        <v>1</v>
-      </c>
-      <c r="J14" s="21">
-        <v>2</v>
-      </c>
-      <c r="K14" s="21">
-        <v>2</v>
-      </c>
-      <c r="L14" s="21">
-        <v>2</v>
-      </c>
-      <c r="M14" s="21">
-        <v>1</v>
-      </c>
-      <c r="N14" s="21">
-        <v>2</v>
-      </c>
-      <c r="O14" s="21">
-        <v>2</v>
-      </c>
-      <c r="P14" s="21">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="21">
-        <v>2</v>
-      </c>
-      <c r="R14" s="21">
-        <v>2</v>
-      </c>
-      <c r="S14" s="21">
-        <v>1</v>
-      </c>
-      <c r="T14" s="21">
-        <v>2</v>
-      </c>
-      <c r="U14" s="21">
-        <v>1</v>
-      </c>
-      <c r="V14" s="21">
-        <v>1</v>
-      </c>
-      <c r="W14" s="21">
-        <v>1</v>
-      </c>
-      <c r="X14" s="21">
-        <v>1</v>
-      </c>
-      <c r="Y14" s="21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
+      <c r="B15" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="E15" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="F15" s="10" t="s">
         <v>209</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>210</v>
       </c>
       <c r="G15" s="10"/>
       <c r="H15" s="10" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I15" s="21">
         <v>1</v>
@@ -3279,7 +3424,7 @@
         <v>1</v>
       </c>
       <c r="K15" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L15" s="21">
         <v>2</v>
@@ -3291,7 +3436,7 @@
         <v>2</v>
       </c>
       <c r="O15" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P15" s="21">
         <v>1</v>
@@ -3300,58 +3445,62 @@
         <v>1</v>
       </c>
       <c r="R15" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S15" s="21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T15" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U15" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V15" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W15" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X15" s="21">
         <v>2</v>
       </c>
       <c r="Y15" s="21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="Z15" s="21">
+        <v>1</v>
+      </c>
+      <c r="AA15" s="21"/>
+    </row>
+    <row r="16" spans="1:27" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="F16" s="7" t="s">
         <v>214</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>215</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I16" s="21">
         <v>2</v>
       </c>
       <c r="J16" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" s="21">
         <v>1</v>
@@ -3360,10 +3509,10 @@
         <v>1</v>
       </c>
       <c r="M16" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N16" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O16" s="21">
         <v>1</v>
@@ -3375,50 +3524,76 @@
         <v>1</v>
       </c>
       <c r="R16" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S16" s="21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T16" s="21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U16" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V16" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W16" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X16" s="21">
         <v>2</v>
       </c>
       <c r="Y16" s="21">
-        <v>0</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="Z16" s="21">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="21"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="22" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y16" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="I2:Y16">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+  <autoFilter ref="A1:Z16" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="J2:Z16">
+    <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
       <formula>2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="10" operator="equal">
+      <formula>"X"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I16">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
+      <formula>"X"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA2:AA16">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"X"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="I2:Y16" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="I2:AA16" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"0,1,2,X"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3442,278 +3617,278 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>219</v>
-      </c>
       <c r="C1" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>223</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>230</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C3" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>236</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="C5" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="D5" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>246</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>246</v>
-      </c>
-      <c r="F5" s="10" t="s">
+      <c r="G5" s="10" t="s">
         <v>247</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>254</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="C7" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="D7" s="10" t="s">
+      <c r="E7" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>258</v>
-      </c>
-      <c r="F7" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>259</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="E8" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>264</v>
-      </c>
       <c r="G8" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="C9" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="C9" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="D9" s="10" t="s">
+      <c r="E9" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>267</v>
-      </c>
-      <c r="F9" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>268</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>273</v>
-      </c>
       <c r="G10" s="7" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="C11" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="D11" s="10" t="s">
+      <c r="E11" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="F11" s="10" t="s">
+      <c r="G11" s="10" t="s">
         <v>277</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>279</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="C12" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>280</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="E12" s="7" t="s">
+      <c r="F12" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>282</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -3737,107 +3912,107 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="24" t="s">
         <v>286</v>
-      </c>
-      <c r="B3" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B4" s="25">
         <v>10000000</v>
       </c>
       <c r="C4" s="18" t="str">
-        <f>INDEX('1. Drivers'!$C$2:$C$5,MATCH(B4,'1. Drivers'!$D$2:$D$5,1))</f>
+        <f>INDEX('1. Drivers'!$C$3:$C$6,MATCH(B4,'1. Drivers'!$D$3:$D$6,1))</f>
         <v>V3 Threshold to £20m</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" s="26">
         <v>40</v>
       </c>
       <c r="C5" s="18" t="str">
-        <f>INDEX('1. Drivers'!$C$6:$C$8,MATCH(B5,'1. Drivers'!$D$6:$D$8,1))</f>
+        <f>INDEX('1. Drivers'!$C$7:$C$9,MATCH(B5,'1. Drivers'!$D$7:$D$9,1))</f>
         <v>D2 27–52 wks</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B6" s="26">
         <v>5</v>
       </c>
       <c r="C6" s="18" t="str">
-        <f>INDEX('1. Drivers'!$C$9:$C$11,MATCH(B6,'1. Drivers'!$D$9:$D$11,1))</f>
+        <f>INDEX('1. Drivers'!$C$10:$C$12,MATCH(B6,'1. Drivers'!$D$10:$D$12,1))</f>
         <v>R3 High</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C7" s="18" t="str">
-        <f>INDEX('1. Drivers'!$C$12:$C$18,MATCH(B7,'1. Drivers'!$E$12:$E$18,0))</f>
+        <f>INDEX('1. Drivers'!$C$13:$C$19,MATCH(B7,'1. Drivers'!$E$13:$E$19,0))</f>
         <v>P2 Fixed/certain final cost</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="24" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B10" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="C10" s="24" t="s">
         <v>292</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="D10" s="24" t="s">
         <v>293</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="E10" s="24" t="s">
+        <v>292</v>
+      </c>
+      <c r="F10" s="24" t="s">
         <v>294</v>
       </c>
-      <c r="E10" s="24" t="s">
-        <v>293</v>
-      </c>
-      <c r="F10" s="24" t="s">
+      <c r="G10" s="24" t="s">
         <v>295</v>
-      </c>
-      <c r="G10" s="24" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="9" t="str">
         <f>IF(INDEX($J$20:$J$23,MATCH(1,$L$20:$L$23,0))&lt;0,"—",INDEX($C$20:$C$23,MATCH(1,$L$20:$L$23,0)))</f>
@@ -3866,7 +4041,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12" s="9" t="str">
         <f>IF(INDEX($J$24:$J$28,MATCH(1,$L$24:$L$28,0))&lt;0,"—",INDEX($C$24:$C$28,MATCH(1,$L$24:$L$28,0)))</f>
@@ -3893,17 +4068,17 @@
         <v>CM1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B13" s="9" t="str">
-        <f>IFERROR(INDEX('3. Contracts'!$C$2:$E$12,MATCH($F$11&amp;"|"&amp;$F$12,'3. Contracts'!$A$2:$A$12,0),MIN(3,MATCH($B$4,'1. Drivers'!$D$2:$D$5,1))),"—")</f>
+        <f>IFERROR(INDEX('3. Contracts'!$C$2:$E$12,MATCH($F$11&amp;"|"&amp;$F$12,'3. Contracts'!$A$2:$A$12,0),MIN(3,MATCH($B$4,'1. Drivers'!$D$3:$D$6,1))),"—")</f>
         <v>JCT Design and Build (DB)</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="9" t="str">
-        <f>IFERROR(INDEX('3. Contracts'!$C$2:$E$12,MATCH($G$11&amp;"|"&amp;$G$12,'3. Contracts'!$A$2:$A$12,0),MIN(3,MATCH($B$4,'1. Drivers'!$D$2:$D$5,1))),"—")</f>
+        <f>IFERROR(INDEX('3. Contracts'!$C$2:$E$12,MATCH($G$11&amp;"|"&amp;$G$12,'3. Contracts'!$A$2:$A$12,0),MIN(3,MATCH($B$4,'1. Drivers'!$D$3:$D$6,1))),"—")</f>
         <v>JCT Standard Building Contract with Quantities (SBC/Q) or without Quantities (SBC/XQ)</v>
       </c>
       <c r="E13" s="10"/>
@@ -3912,7 +4087,7 @@
     </row>
     <row r="14" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B14" s="9" t="str">
         <f>IFERROR(INDEX('3. Contracts'!$F$2:$F$12,MATCH($F$11&amp;"|"&amp;$F$12,'3. Contracts'!$A$2:$A$12,0)),"—")</f>
@@ -3929,7 +4104,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15" s="9" t="str">
         <f>IF(INDEX($J$29:$J$34,MATCH(1,$L$29:$L$34,0))&lt;0,"—",INDEX($C$29:$C$34,MATCH(1,$L$29:$L$34,0)))</f>
@@ -3958,54 +4133,54 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="22" t="str">
-        <f>"Maximum score: "&amp;(2*('1. Drivers'!$D$21+'1. Drivers'!$D$22+'1. Drivers'!$D$23+'1. Drivers'!$D$24))&amp;". Commercial model and contract in the Alternative column go with the alternative route."</f>
+        <f>"Maximum score: "&amp;(2*('1. Drivers'!$D$22+'1. Drivers'!$D$23+'1. Drivers'!$D$24+'1. Drivers'!$D$25))&amp;". Commercial model and contract in the Alternative column go with the alternative route."</f>
         <v>Maximum score: 10. Commercial model and contract in the Alternative column go with the alternative route.</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>129</v>
-      </c>
       <c r="D19" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G19" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="H19" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="I19" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="J19" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="I19" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="J19" s="5" t="s">
+      <c r="K19" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="K19" s="5" t="s">
+      <c r="L19" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="L19" s="5" t="s">
+      <c r="M19" s="5" t="s">
         <v>304</v>
-      </c>
-      <c r="M19" s="5" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -4022,19 +4197,19 @@
         <v>Traditional</v>
       </c>
       <c r="D20" s="21">
-        <f>INDEX('2. Options'!$I2:$L2,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J2:$M2,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>1</v>
       </c>
       <c r="E20" s="21">
-        <f>INDEX('2. Options'!$M2:$O2,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N2:$P2,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>2</v>
       </c>
       <c r="F20" s="21">
-        <f>INDEX('2. Options'!$P2:$R2,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q2:$S2,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>0</v>
       </c>
       <c r="G20" s="21">
-        <f>INDEX('2. Options'!$S2:$Y2,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T2:$Z2,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>2</v>
       </c>
       <c r="H20" s="21" t="str">
@@ -4042,7 +4217,7 @@
         <v>No</v>
       </c>
       <c r="I20" s="21">
-        <f>IF(H20="Yes","",D20*'1. Drivers'!$D$21+E20*'1. Drivers'!$D$22+F20*'1. Drivers'!$D$23+G20*'1. Drivers'!$D$24)</f>
+        <f>IF(H20="Yes","",D20*'1. Drivers'!$D$22+E20*'1. Drivers'!$D$23+F20*'1. Drivers'!$D$24+G20*'1. Drivers'!$D$25)</f>
         <v>7</v>
       </c>
       <c r="J20" s="29">
@@ -4076,19 +4251,19 @@
         <v>Design and build (single stage)</v>
       </c>
       <c r="D21" s="21">
-        <f>INDEX('2. Options'!$I3:$L3,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J3:$M3,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>2</v>
       </c>
       <c r="E21" s="21">
-        <f>INDEX('2. Options'!$M3:$O3,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N3:$P3,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>2</v>
       </c>
       <c r="F21" s="21">
-        <f>INDEX('2. Options'!$P3:$R3,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q3:$S3,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>1</v>
       </c>
       <c r="G21" s="21">
-        <f>INDEX('2. Options'!$S3:$Y3,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T3:$Z3,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>2</v>
       </c>
       <c r="H21" s="21" t="str">
@@ -4096,7 +4271,7 @@
         <v>No</v>
       </c>
       <c r="I21" s="21">
-        <f>IF(H21="Yes","",D21*'1. Drivers'!$D$21+E21*'1. Drivers'!$D$22+F21*'1. Drivers'!$D$23+G21*'1. Drivers'!$D$24)</f>
+        <f>IF(H21="Yes","",D21*'1. Drivers'!$D$22+E21*'1. Drivers'!$D$23+F21*'1. Drivers'!$D$24+G21*'1. Drivers'!$D$25)</f>
         <v>9</v>
       </c>
       <c r="J21" s="29">
@@ -4130,19 +4305,19 @@
         <v>Two-stage (PCSA)</v>
       </c>
       <c r="D22" s="21">
-        <f>INDEX('2. Options'!$I4:$L4,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J4:$M4,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>2</v>
       </c>
       <c r="E22" s="21">
-        <f>INDEX('2. Options'!$M4:$O4,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N4:$P4,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>1</v>
       </c>
       <c r="F22" s="21">
-        <f>INDEX('2. Options'!$P4:$R4,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q4:$S4,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>2</v>
       </c>
       <c r="G22" s="21">
-        <f>INDEX('2. Options'!$S4:$Y4,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T4:$Z4,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>1</v>
       </c>
       <c r="H22" s="21" t="str">
@@ -4150,7 +4325,7 @@
         <v>No</v>
       </c>
       <c r="I22" s="21">
-        <f>IF(H22="Yes","",D22*'1. Drivers'!$D$21+E22*'1. Drivers'!$D$22+F22*'1. Drivers'!$D$23+G22*'1. Drivers'!$D$24)</f>
+        <f>IF(H22="Yes","",D22*'1. Drivers'!$D$22+E22*'1. Drivers'!$D$23+F22*'1. Drivers'!$D$24+G22*'1. Drivers'!$D$25)</f>
         <v>7</v>
       </c>
       <c r="J22" s="29">
@@ -4184,19 +4359,19 @@
         <v>Construction management</v>
       </c>
       <c r="D23" s="21">
-        <f>INDEX('2. Options'!$I5:$L5,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J5:$M5,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>0</v>
       </c>
       <c r="E23" s="21">
-        <f>INDEX('2. Options'!$M5:$O5,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N5:$P5,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>1</v>
       </c>
       <c r="F23" s="21">
-        <f>INDEX('2. Options'!$P5:$R5,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q5:$S5,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>2</v>
       </c>
       <c r="G23" s="21">
-        <f>INDEX('2. Options'!$S5:$Y5,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T5:$Z5,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>0</v>
       </c>
       <c r="H23" s="21" t="str">
@@ -4204,7 +4379,7 @@
         <v>No</v>
       </c>
       <c r="I23" s="21">
-        <f>IF(H23="Yes","",D23*'1. Drivers'!$D$21+E23*'1. Drivers'!$D$22+F23*'1. Drivers'!$D$23+G23*'1. Drivers'!$D$24)</f>
+        <f>IF(H23="Yes","",D23*'1. Drivers'!$D$22+E23*'1. Drivers'!$D$23+F23*'1. Drivers'!$D$24+G23*'1. Drivers'!$D$25)</f>
         <v>3</v>
       </c>
       <c r="J23" s="29">
@@ -4238,19 +4413,19 @@
         <v>Lump sum</v>
       </c>
       <c r="D24" s="21">
-        <f>INDEX('2. Options'!$I6:$L6,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J6:$M6,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>2</v>
       </c>
       <c r="E24" s="21">
-        <f>INDEX('2. Options'!$M6:$O6,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N6:$P6,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>2</v>
       </c>
       <c r="F24" s="21">
-        <f>INDEX('2. Options'!$P6:$R6,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q6:$S6,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>0</v>
       </c>
       <c r="G24" s="21">
-        <f>INDEX('2. Options'!$S6:$Y6,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T6:$Z6,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>2</v>
       </c>
       <c r="H24" s="21" t="str">
@@ -4258,7 +4433,7 @@
         <v>No</v>
       </c>
       <c r="I24" s="21">
-        <f>IF(H24="Yes","",D24*'1. Drivers'!$D$21+E24*'1. Drivers'!$D$22+F24*'1. Drivers'!$D$23+G24*'1. Drivers'!$D$24)</f>
+        <f>IF(H24="Yes","",D24*'1. Drivers'!$D$22+E24*'1. Drivers'!$D$23+F24*'1. Drivers'!$D$24+G24*'1. Drivers'!$D$25)</f>
         <v>8</v>
       </c>
       <c r="J24" s="29">
@@ -4292,19 +4467,19 @@
         <v>Guaranteed maximum price (GMP)</v>
       </c>
       <c r="D25" s="21">
-        <f>INDEX('2. Options'!$I7:$L7,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J7:$M7,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>2</v>
       </c>
       <c r="E25" s="21">
-        <f>INDEX('2. Options'!$M7:$O7,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N7:$P7,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>1</v>
       </c>
       <c r="F25" s="21">
-        <f>INDEX('2. Options'!$P7:$R7,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q7:$S7,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>1</v>
       </c>
       <c r="G25" s="21">
-        <f>INDEX('2. Options'!$S7:$Y7,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T7:$Z7,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>2</v>
       </c>
       <c r="H25" s="21" t="str">
@@ -4312,7 +4487,7 @@
         <v>No</v>
       </c>
       <c r="I25" s="21">
-        <f>IF(H25="Yes","",D25*'1. Drivers'!$D$21+E25*'1. Drivers'!$D$22+F25*'1. Drivers'!$D$23+G25*'1. Drivers'!$D$24)</f>
+        <f>IF(H25="Yes","",D25*'1. Drivers'!$D$22+E25*'1. Drivers'!$D$23+F25*'1. Drivers'!$D$24+G25*'1. Drivers'!$D$25)</f>
         <v>8</v>
       </c>
       <c r="J25" s="29">
@@ -4346,19 +4521,19 @@
         <v>Target cost</v>
       </c>
       <c r="D26" s="21">
-        <f>INDEX('2. Options'!$I8:$L8,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J8:$M8,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>2</v>
       </c>
       <c r="E26" s="21">
-        <f>INDEX('2. Options'!$M8:$O8,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N8:$P8,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>1</v>
       </c>
       <c r="F26" s="21">
-        <f>INDEX('2. Options'!$P8:$R8,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q8:$S8,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>2</v>
       </c>
       <c r="G26" s="21">
-        <f>INDEX('2. Options'!$S8:$Y8,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T8:$Z8,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>0</v>
       </c>
       <c r="H26" s="21" t="str">
@@ -4366,7 +4541,7 @@
         <v>No</v>
       </c>
       <c r="I26" s="21">
-        <f>IF(H26="Yes","",D26*'1. Drivers'!$D$21+E26*'1. Drivers'!$D$22+F26*'1. Drivers'!$D$23+G26*'1. Drivers'!$D$24)</f>
+        <f>IF(H26="Yes","",D26*'1. Drivers'!$D$22+E26*'1. Drivers'!$D$23+F26*'1. Drivers'!$D$24+G26*'1. Drivers'!$D$25)</f>
         <v>5</v>
       </c>
       <c r="J26" s="29">
@@ -4400,19 +4575,19 @@
         <v>Remeasurement</v>
       </c>
       <c r="D27" s="21">
-        <f>INDEX('2. Options'!$I9:$L9,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J9:$M9,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>1</v>
       </c>
       <c r="E27" s="21">
-        <f>INDEX('2. Options'!$M9:$O9,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N9:$P9,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>2</v>
       </c>
       <c r="F27" s="21">
-        <f>INDEX('2. Options'!$P9:$R9,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q9:$S9,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>2</v>
       </c>
       <c r="G27" s="21">
-        <f>INDEX('2. Options'!$S9:$Y9,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T9:$Z9,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>0</v>
       </c>
       <c r="H27" s="21" t="str">
@@ -4420,7 +4595,7 @@
         <v>No</v>
       </c>
       <c r="I27" s="21">
-        <f>IF(H27="Yes","",D27*'1. Drivers'!$D$21+E27*'1. Drivers'!$D$22+F27*'1. Drivers'!$D$23+G27*'1. Drivers'!$D$24)</f>
+        <f>IF(H27="Yes","",D27*'1. Drivers'!$D$22+E27*'1. Drivers'!$D$23+F27*'1. Drivers'!$D$24+G27*'1. Drivers'!$D$25)</f>
         <v>5</v>
       </c>
       <c r="J27" s="29">
@@ -4454,19 +4629,19 @@
         <v>Cost reimbursable</v>
       </c>
       <c r="D28" s="21">
-        <f>INDEX('2. Options'!$I10:$L10,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J10:$M10,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>0</v>
       </c>
       <c r="E28" s="21">
-        <f>INDEX('2. Options'!$M10:$O10,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N10:$P10,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>1</v>
       </c>
       <c r="F28" s="21">
-        <f>INDEX('2. Options'!$P10:$R10,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q10:$S10,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>2</v>
       </c>
       <c r="G28" s="21">
-        <f>INDEX('2. Options'!$S10:$Y10,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T10:$Z10,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>0</v>
       </c>
       <c r="H28" s="21" t="str">
@@ -4474,7 +4649,7 @@
         <v>No</v>
       </c>
       <c r="I28" s="21">
-        <f>IF(H28="Yes","",D28*'1. Drivers'!$D$21+E28*'1. Drivers'!$D$22+F28*'1. Drivers'!$D$23+G28*'1. Drivers'!$D$24)</f>
+        <f>IF(H28="Yes","",D28*'1. Drivers'!$D$22+E28*'1. Drivers'!$D$23+F28*'1. Drivers'!$D$24+G28*'1. Drivers'!$D$25)</f>
         <v>3</v>
       </c>
       <c r="J28" s="29">
@@ -4508,19 +4683,19 @@
         <v>Quotations</v>
       </c>
       <c r="D29" s="21" t="str">
-        <f>INDEX('2. Options'!$I11:$L11,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J11:$M11,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>X</v>
       </c>
       <c r="E29" s="21">
-        <f>INDEX('2. Options'!$M11:$O11,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N11:$P11,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>1</v>
       </c>
       <c r="F29" s="21">
-        <f>INDEX('2. Options'!$P11:$R11,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q11:$S11,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>0</v>
       </c>
       <c r="G29" s="21">
-        <f>INDEX('2. Options'!$S11:$Y11,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T11:$Z11,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>1</v>
       </c>
       <c r="H29" s="21" t="str">
@@ -4528,7 +4703,7 @@
         <v>Yes</v>
       </c>
       <c r="I29" s="21" t="str">
-        <f>IF(H29="Yes","",D29*'1. Drivers'!$D$21+E29*'1. Drivers'!$D$22+F29*'1. Drivers'!$D$23+G29*'1. Drivers'!$D$24)</f>
+        <f>IF(H29="Yes","",D29*'1. Drivers'!$D$22+E29*'1. Drivers'!$D$23+F29*'1. Drivers'!$D$24+G29*'1. Drivers'!$D$25)</f>
         <v/>
       </c>
       <c r="J29" s="29">
@@ -4562,19 +4737,19 @@
         <v>Open tender</v>
       </c>
       <c r="D30" s="21">
-        <f>INDEX('2. Options'!$I12:$L12,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J12:$M12,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>2</v>
       </c>
       <c r="E30" s="21">
-        <f>INDEX('2. Options'!$M12:$O12,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N12:$P12,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>1</v>
       </c>
       <c r="F30" s="21">
-        <f>INDEX('2. Options'!$P12:$R12,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q12:$S12,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>0</v>
       </c>
       <c r="G30" s="21">
-        <f>INDEX('2. Options'!$S12:$Y12,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T12:$Z12,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>2</v>
       </c>
       <c r="H30" s="21" t="str">
@@ -4582,7 +4757,7 @@
         <v>No</v>
       </c>
       <c r="I30" s="21">
-        <f>IF(H30="Yes","",D30*'1. Drivers'!$D$21+E30*'1. Drivers'!$D$22+F30*'1. Drivers'!$D$23+G30*'1. Drivers'!$D$24)</f>
+        <f>IF(H30="Yes","",D30*'1. Drivers'!$D$22+E30*'1. Drivers'!$D$23+F30*'1. Drivers'!$D$24+G30*'1. Drivers'!$D$25)</f>
         <v>7</v>
       </c>
       <c r="J30" s="29">
@@ -4616,19 +4791,19 @@
         <v>Selective tender</v>
       </c>
       <c r="D31" s="21">
-        <f>INDEX('2. Options'!$I13:$L13,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J13:$M13,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>1</v>
       </c>
       <c r="E31" s="21">
-        <f>INDEX('2. Options'!$M13:$O13,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N13:$P13,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>2</v>
       </c>
       <c r="F31" s="21">
-        <f>INDEX('2. Options'!$P13:$R13,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q13:$S13,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>1</v>
       </c>
       <c r="G31" s="21">
-        <f>INDEX('2. Options'!$S13:$Y13,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T13:$Z13,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>2</v>
       </c>
       <c r="H31" s="21" t="str">
@@ -4636,7 +4811,7 @@
         <v>No</v>
       </c>
       <c r="I31" s="21">
-        <f>IF(H31="Yes","",D31*'1. Drivers'!$D$21+E31*'1. Drivers'!$D$22+F31*'1. Drivers'!$D$23+G31*'1. Drivers'!$D$24)</f>
+        <f>IF(H31="Yes","",D31*'1. Drivers'!$D$22+E31*'1. Drivers'!$D$23+F31*'1. Drivers'!$D$24+G31*'1. Drivers'!$D$25)</f>
         <v>8</v>
       </c>
       <c r="J31" s="29">
@@ -4670,19 +4845,19 @@
         <v>Framework — mini-competition</v>
       </c>
       <c r="D32" s="21">
-        <f>INDEX('2. Options'!$I14:$L14,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J14:$M14,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>2</v>
       </c>
       <c r="E32" s="21">
-        <f>INDEX('2. Options'!$M14:$O14,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N14:$P14,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>2</v>
       </c>
       <c r="F32" s="21">
-        <f>INDEX('2. Options'!$P14:$R14,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q14:$S14,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>2</v>
       </c>
       <c r="G32" s="21">
-        <f>INDEX('2. Options'!$S14:$Y14,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T14:$Z14,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>2</v>
       </c>
       <c r="H32" s="21" t="str">
@@ -4690,7 +4865,7 @@
         <v>Yes</v>
       </c>
       <c r="I32" s="21" t="str">
-        <f>IF(H32="Yes","",D32*'1. Drivers'!$D$21+E32*'1. Drivers'!$D$22+F32*'1. Drivers'!$D$23+G32*'1. Drivers'!$D$24)</f>
+        <f>IF(H32="Yes","",D32*'1. Drivers'!$D$22+E32*'1. Drivers'!$D$23+F32*'1. Drivers'!$D$24+G32*'1. Drivers'!$D$25)</f>
         <v/>
       </c>
       <c r="J32" s="29">
@@ -4724,19 +4899,19 @@
         <v>Framework — direct award</v>
       </c>
       <c r="D33" s="21">
-        <f>INDEX('2. Options'!$I15:$L15,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J15:$M15,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>2</v>
       </c>
       <c r="E33" s="21">
-        <f>INDEX('2. Options'!$M15:$O15,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N15:$P15,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>2</v>
       </c>
       <c r="F33" s="21">
-        <f>INDEX('2. Options'!$P15:$R15,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q15:$S15,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>2</v>
       </c>
       <c r="G33" s="21">
-        <f>INDEX('2. Options'!$S15:$Y15,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T15:$Z15,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>1</v>
       </c>
       <c r="H33" s="21" t="str">
@@ -4744,7 +4919,7 @@
         <v>Yes</v>
       </c>
       <c r="I33" s="21" t="str">
-        <f>IF(H33="Yes","",D33*'1. Drivers'!$D$21+E33*'1. Drivers'!$D$22+F33*'1. Drivers'!$D$23+G33*'1. Drivers'!$D$24)</f>
+        <f>IF(H33="Yes","",D33*'1. Drivers'!$D$22+E33*'1. Drivers'!$D$23+F33*'1. Drivers'!$D$24+G33*'1. Drivers'!$D$25)</f>
         <v/>
       </c>
       <c r="J33" s="29">
@@ -4778,19 +4953,19 @@
         <v>Negotiated</v>
       </c>
       <c r="D34" s="21">
-        <f>INDEX('2. Options'!$I16:$L16,1,MATCH($C$4,'2. Options'!$I$1:$L$1,0))</f>
+        <f>INDEX('2. Options'!$J16:$M16,1,MATCH($C$4,'2. Options'!$J$1:$M$1,0))</f>
         <v>1</v>
       </c>
       <c r="E34" s="21">
-        <f>INDEX('2. Options'!$M16:$O16,1,MATCH($C$5,'2. Options'!$M$1:$O$1,0))</f>
+        <f>INDEX('2. Options'!$N16:$P16,1,MATCH($C$5,'2. Options'!$N$1:$P$1,0))</f>
         <v>1</v>
       </c>
       <c r="F34" s="21">
-        <f>INDEX('2. Options'!$P16:$R16,1,MATCH($C$6,'2. Options'!$P$1:$R$1,0))</f>
+        <f>INDEX('2. Options'!$Q16:$S16,1,MATCH($C$6,'2. Options'!$Q$1:$S$1,0))</f>
         <v>2</v>
       </c>
       <c r="G34" s="21">
-        <f>INDEX('2. Options'!$S16:$Y16,1,MATCH($C$7,'2. Options'!$S$1:$Y$1,0))</f>
+        <f>INDEX('2. Options'!$T16:$Z16,1,MATCH($C$7,'2. Options'!$T$1:$Z$1,0))</f>
         <v>1</v>
       </c>
       <c r="H34" s="21" t="str">
@@ -4798,7 +4973,7 @@
         <v>No</v>
       </c>
       <c r="I34" s="21">
-        <f>IF(H34="Yes","",D34*'1. Drivers'!$D$21+E34*'1. Drivers'!$D$22+F34*'1. Drivers'!$D$23+G34*'1. Drivers'!$D$24)</f>
+        <f>IF(H34="Yes","",D34*'1. Drivers'!$D$22+E34*'1. Drivers'!$D$23+F34*'1. Drivers'!$D$24+G34*'1. Drivers'!$D$25)</f>
         <v>6</v>
       </c>
       <c r="J34" s="29">
@@ -4832,7 +5007,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0400-000000000000}">
           <x14:formula1>
-            <xm:f>'1. Drivers'!$E$12:$E$18</xm:f>
+            <xm:f>'1. Drivers'!$E$13:$E$19</xm:f>
           </x14:formula1>
           <x14:formula2>
             <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Procurement Reference v2.2: tab 5 'Routes and contracts' (RIBA Plan of Work 2020); procurement-programme brief
Reference tab only: the four RIBA routes (Traditional, Design & Build 1
Stage, Design & Build 2 Stage, Management Contract / Construction
Management) and the contracts within each - JCT MW / MWD and NEC4 ECS for
small simple work, the CDP option (ICD, SBC + CDP) under Traditional, and
the D&B, PCSA and management forms - with when the contractor comes in and
the programme effect. Owner's decisions (11 Oct 2026): Minor Works up to
1m, no overlap of Stage 4 and construction, Contractor-led not offered.
Tabs 1-3 unchanged; the app does not read tab 5 yet.

docs/procurement-programme-brief-2026-10-11.md is the plan for the engine.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Projento_Procurement_Reference.xlsx
+++ b/Projento_Procurement_Reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\estates-ai-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0250CFB5-F4BC-484F-B409-DCBDCE876166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB531D20-D86D-489E-8DCE-FDBEC5048B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2250" yWindow="2250" windowWidth="21600" windowHeight="11295" tabRatio="500" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Read Me" sheetId="1" r:id="rId1"/>
@@ -18,11 +18,12 @@
     <sheet name="2. Options" sheetId="3" r:id="rId3"/>
     <sheet name="3. Contracts" sheetId="4" r:id="rId4"/>
     <sheet name="4. Check" sheetId="5" r:id="rId5"/>
+    <sheet name="5. Routes and contracts" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. Options'!$A$1:$Z$16</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1" calcId="191029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="386">
   <si>
     <t>Projento — Procurement Reference v2</t>
   </si>
@@ -713,9 +714,6 @@
     <t>Route + commercial model</t>
   </si>
   <si>
-    <t>JCT — V1 under £1m</t>
-  </si>
-  <si>
     <t>JCT — V2 £1m to threshold</t>
   </si>
   <si>
@@ -986,10 +984,235 @@
     <t>External works only</t>
   </si>
   <si>
-    <t>2.1 · 10 October 2026 · Nabil Kayali · replaces v2.0 (value level V0 under £100k; Quotations only under £100k; Project types column — Remeasurement for External works only)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JCT — V0/V1 under £1m</t>
+    <t>JCT — V0/V1 under £1m</t>
+  </si>
+  <si>
+    <t>PROCUREMENT ROUTES AND THEIR CONTRACTS — RIBA Plan of Work 2020</t>
+  </si>
+  <si>
+    <t>The route decides WHEN the contractor is brought in and who designs; the contract is chosen WITHIN the route; the route to market (tab 2) decides how long the tender takes. Reference for the owner; the app does not read this tab yet (see docs/procurement-programme-brief-2026-10-11.md).</t>
+  </si>
+  <si>
+    <t>Route (RIBA)</t>
+  </si>
+  <si>
+    <t>Contractor brought in</t>
+  </si>
+  <si>
+    <t>Contract</t>
+  </si>
+  <si>
+    <t>Form</t>
+  </si>
+  <si>
+    <t>Use it when</t>
+  </si>
+  <si>
+    <t>Programme effect</t>
+  </si>
+  <si>
+    <t>Tender at the end of Stage 4</t>
+  </si>
+  <si>
+    <t>Minor Works Building Contract (MW)</t>
+  </si>
+  <si>
+    <t>JCT</t>
+  </si>
+  <si>
+    <t>Simple work fully designed by the client's team; refurbishment, fit-out or external works; no specialist design</t>
+  </si>
+  <si>
+    <t>Up to £1m</t>
+  </si>
+  <si>
+    <t>Stage 3 and Stage 4 combined into one short design-and-specification stage</t>
+  </si>
+  <si>
+    <t>Minor Works with Contractor's Design (MWD)</t>
+  </si>
+  <si>
+    <t>As MW, where the contractor designs one named part (e.g. ventilation)</t>
+  </si>
+  <si>
+    <t>As MW</t>
+  </si>
+  <si>
+    <t>Engineering and Construction Short Contract (ECS)</t>
+  </si>
+  <si>
+    <t>NEC4</t>
+  </si>
+  <si>
+    <t>Simple, low-risk work (NEC4 equivalent of MW)</t>
+  </si>
+  <si>
+    <t>Intermediate Building Contract (IC)</t>
+  </si>
+  <si>
+    <t>Medium-sized work fully designed by the client's team</t>
+  </si>
+  <si>
+    <t>£1m to threshold</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Intermediate with Contractor's Design (ICD) — CDP option</t>
+  </si>
+  <si>
+    <t>As IC, where the contractor designs named parts (services, cladding, roofing systems)</t>
+  </si>
+  <si>
+    <t>Client's Stage 4 shorter (named parts by performance specification)</t>
+  </si>
+  <si>
+    <t>Standard Building Contract with / without Quantities (SBC)</t>
+  </si>
+  <si>
+    <t>Large or complex work fully designed by the client</t>
+  </si>
+  <si>
+    <t>Above threshold</t>
+  </si>
+  <si>
+    <t>Standard Building Contract with Contractor's Designed Portion (SBC + CDP) — CDP option</t>
+  </si>
+  <si>
+    <t>As SBC, where the contractor designs named parts</t>
+  </si>
+  <si>
+    <t>Client's Stage 4 shorter</t>
+  </si>
+  <si>
+    <t>Engineering and Construction Contract (ECC) Option A or B</t>
+  </si>
+  <si>
+    <t>Priced contract with activity schedule (A) or bill of quantities (B)</t>
+  </si>
+  <si>
+    <t>Any</t>
+  </si>
+  <si>
+    <t>Measured Term Contract (MTC) / Prime Cost (PCC)</t>
+  </si>
+  <si>
+    <t>Repeat or term works (MTC); urgent or undefined work (PCC)</t>
+  </si>
+  <si>
+    <t>Design &amp; Build 1 Stage</t>
+  </si>
+  <si>
+    <t>Employer's Requirements at the end of Stage 3; contractor appointed at the start of Stage 4</t>
+  </si>
+  <si>
+    <t>Design and Build Contract (DB)</t>
+  </si>
+  <si>
+    <t>Client can state clear requirements; one point of responsibility</t>
+  </si>
+  <si>
+    <t>£1m and above</t>
+  </si>
+  <si>
+    <t>Tender after Stage 3; the contractor does Stage 4 after award, then builds</t>
+  </si>
+  <si>
+    <t>Employer's Requirements at the end of Stage 3</t>
+  </si>
+  <si>
+    <t>Small design and build work</t>
+  </si>
+  <si>
+    <t>As DB</t>
+  </si>
+  <si>
+    <t>NEC4 equivalent of DB</t>
+  </si>
+  <si>
+    <t>Design &amp; Build 2 Stage</t>
+  </si>
+  <si>
+    <t>Employer's Requirements at the end of Stage 2; contractor under a PCSA through Stage 3; price agreed and appointed at the start of Stage 4</t>
+  </si>
+  <si>
+    <t>Pre-Construction Services Agreement (PCSA), then DB or Constructing Excellence (CE)</t>
+  </si>
+  <si>
+    <t>Complex or time-critical projects needing early contractor input</t>
+  </si>
+  <si>
+    <t>First-stage tender after Stage 2 alongside Stage 3; second-stage price at the end of Stage 3; contractor does Stage 4, then builds</t>
+  </si>
+  <si>
+    <t>As above</t>
+  </si>
+  <si>
+    <t>NEC4 equivalent, target cost</t>
+  </si>
+  <si>
+    <t>Management Contract / Construction Management</t>
+  </si>
+  <si>
+    <t>Contractor appointed at the end of Stage 2</t>
+  </si>
+  <si>
+    <t>Management Building Contract (MC) / Construction Management Appointment + trade contracts</t>
+  </si>
+  <si>
+    <t>Large, complex projects designed and let package by package</t>
+  </si>
+  <si>
+    <t>Appointment after Stage 2 alongside Stage 3; packages tendered during Stage 4; site work after Stage 4</t>
+  </si>
+  <si>
+    <t>ECC Option F (management contract)</t>
+  </si>
+  <si>
+    <t>WHEN MINOR WORKS (MW / MWD / ECS) IS SUGGESTED — all must hold</t>
+  </si>
+  <si>
+    <t>Project type</t>
+  </si>
+  <si>
+    <t>Refurbishment, Fit-out or External works only</t>
+  </si>
+  <si>
+    <t>Construction cost under £1m (owner, 11 Oct 2026)</t>
+  </si>
+  <si>
+    <t>Level of work</t>
+  </si>
+  <si>
+    <t>Not "Reconfiguration or full redesign"</t>
+  </si>
+  <si>
+    <t>Specialist design</t>
+  </si>
+  <si>
+    <t>None of: laboratory, clinical, cleanroom, medical gases, fume extraction, lifts, sprinklers, smoke ventilation (one such item on a small job: MWD)</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Up to 500 m² (owner to confirm)</t>
+  </si>
+  <si>
+    <t>Client preference</t>
+  </si>
+  <si>
+    <t>Favoured when the top priority (Q4.4) is Lowest cost or Speed</t>
+  </si>
+  <si>
+    <t>No overlap</t>
+  </si>
+  <si>
+    <t>Owner (11 Oct 2026): work on site starts only when Stage 4 is complete, on every route. Contractor-led is not offered.</t>
+  </si>
+  <si>
+    <t>2.2 · 11 October 2026 · Nabil Kayali · replaces v2.1 (new tab 5 Routes and contracts: the four RIBA Plan of Work 2020 routes and the contracts within each, incl. JCT Minor Works / MWD / NEC4 ECS and the CDP option under Traditional; reference only, the app does not read it yet). Scores, options and contracts in tabs 1–3 unchanged.</t>
   </si>
 </sst>
 </file>
@@ -1000,7 +1223,7 @@
     <numFmt numFmtId="164" formatCode="\£#,##0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1057,8 +1280,22 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1083,6 +1320,12 @@
         <bgColor rgb="FFFFFF99"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A2E4A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1105,7 +1348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1168,61 +1411,19 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF8D7D3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD5E8D4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF8D7D3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD5E8D4"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <b/>
@@ -1521,12 +1722,12 @@
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>310</v>
+        <v>385</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -1835,10 +2036,10 @@
         <v>5</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>306</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>307</v>
       </c>
       <c r="D2" s="8">
         <v>0</v>
@@ -2298,7 +2499,7 @@
         <v>133</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>66</v>
@@ -2352,7 +2553,7 @@
         <v>113</v>
       </c>
       <c r="AA1" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="38.25" x14ac:dyDescent="0.25">
@@ -2994,7 +3195,7 @@
         <v>1</v>
       </c>
       <c r="AA9" s="21" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" spans="1:27" ht="25.5" x14ac:dyDescent="0.25">
@@ -3559,29 +3760,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:Z16" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="J2:Z16">
-    <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
-      <formula>2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="10" operator="equal">
-      <formula>"X"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I16">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
-      <formula>2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
-      <formula>"X"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA2:AA16">
+  <conditionalFormatting sqref="I2:AA16">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>2</formula>
     </cfRule>
@@ -3623,272 +3802,272 @@
         <v>218</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>222</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>229</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C3" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>235</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>241</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="C5" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="D5" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="F5" s="10" t="s">
+      <c r="G5" s="10" t="s">
         <v>246</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>253</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="C7" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="D7" s="10" t="s">
+      <c r="E7" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>257</v>
-      </c>
-      <c r="F7" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>258</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>260</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="E8" s="7" t="s">
-        <v>262</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>263</v>
-      </c>
       <c r="G8" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="C9" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="C9" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="D9" s="10" t="s">
+      <c r="E9" s="10" t="s">
+        <v>265</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>266</v>
-      </c>
-      <c r="F9" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>267</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>272</v>
-      </c>
       <c r="G10" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="C11" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="D11" s="10" t="s">
+      <c r="E11" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>275</v>
-      </c>
-      <c r="F11" s="10" t="s">
+      <c r="G11" s="10" t="s">
         <v>276</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>278</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="C12" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>279</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="E12" s="7" t="s">
+      <c r="F12" s="7" t="s">
         <v>280</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>281</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -3912,28 +4091,28 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B3" s="24" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B4" s="25">
         <v>10000000</v>
@@ -3957,7 +4136,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B6" s="26">
         <v>5</v>
@@ -3969,7 +4148,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B7" s="27" t="s">
         <v>99</v>
@@ -3981,10 +4160,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -3992,22 +4171,22 @@
         <v>127</v>
       </c>
       <c r="B10" s="24" t="s">
+        <v>290</v>
+      </c>
+      <c r="C10" s="24" t="s">
         <v>291</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="D10" s="24" t="s">
         <v>292</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="E10" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="F10" s="24" t="s">
         <v>293</v>
       </c>
-      <c r="E10" s="24" t="s">
-        <v>292</v>
-      </c>
-      <c r="F10" s="24" t="s">
+      <c r="G10" s="24" t="s">
         <v>294</v>
-      </c>
-      <c r="G10" s="24" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -4070,7 +4249,7 @@
     </row>
     <row r="13" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B13" s="9" t="str">
         <f>IFERROR(INDEX('3. Contracts'!$C$2:$E$12,MATCH($F$11&amp;"|"&amp;$F$12,'3. Contracts'!$A$2:$A$12,0),MIN(3,MATCH($B$4,'1. Drivers'!$D$3:$D$6,1))),"—")</f>
@@ -4087,7 +4266,7 @@
     </row>
     <row r="14" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B14" s="9" t="str">
         <f>IFERROR(INDEX('3. Contracts'!$F$2:$F$12,MATCH($F$11&amp;"|"&amp;$F$12,'3. Contracts'!$A$2:$A$12,0)),"—")</f>
@@ -4139,7 +4318,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4162,25 +4341,25 @@
         <v>9</v>
       </c>
       <c r="G19" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="H19" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="I19" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="J19" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="I19" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="J19" s="5" t="s">
+      <c r="K19" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="K19" s="5" t="s">
+      <c r="L19" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="L19" s="5" t="s">
+      <c r="M19" s="5" t="s">
         <v>303</v>
-      </c>
-      <c r="M19" s="5" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -5018,4 +5197,544 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58E248C4-12DC-4602-B3F1-74D2B9672822}">
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="40.7109375" customWidth="1"/>
+    <col min="3" max="3" width="46.7109375" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" customWidth="1"/>
+    <col min="5" max="5" width="50.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="50.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="30" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="31" t="s">
+        <v>312</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>314</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>315</v>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>316</v>
+      </c>
+      <c r="F4" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="31" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>319</v>
+      </c>
+      <c r="D5" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>321</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>322</v>
+      </c>
+      <c r="G5" s="32" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>324</v>
+      </c>
+      <c r="D6" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E6" s="32" t="s">
+        <v>325</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>322</v>
+      </c>
+      <c r="G6" s="32" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>327</v>
+      </c>
+      <c r="D7" s="32" t="s">
+        <v>328</v>
+      </c>
+      <c r="E7" s="32" t="s">
+        <v>329</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>322</v>
+      </c>
+      <c r="G7" s="32" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>330</v>
+      </c>
+      <c r="D8" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E8" s="32" t="s">
+        <v>331</v>
+      </c>
+      <c r="F8" s="32" t="s">
+        <v>332</v>
+      </c>
+      <c r="G8" s="32" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>334</v>
+      </c>
+      <c r="D9" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>335</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>332</v>
+      </c>
+      <c r="G9" s="32" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>337</v>
+      </c>
+      <c r="D10" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E10" s="32" t="s">
+        <v>338</v>
+      </c>
+      <c r="F10" s="32" t="s">
+        <v>339</v>
+      </c>
+      <c r="G10" s="32" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>340</v>
+      </c>
+      <c r="D11" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E11" s="32" t="s">
+        <v>341</v>
+      </c>
+      <c r="F11" s="32" t="s">
+        <v>339</v>
+      </c>
+      <c r="G11" s="32" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>343</v>
+      </c>
+      <c r="D12" s="32" t="s">
+        <v>328</v>
+      </c>
+      <c r="E12" s="32" t="s">
+        <v>344</v>
+      </c>
+      <c r="F12" s="32" t="s">
+        <v>345</v>
+      </c>
+      <c r="G12" s="32" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" s="32" t="s">
+        <v>318</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>346</v>
+      </c>
+      <c r="D13" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E13" s="32" t="s">
+        <v>347</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>345</v>
+      </c>
+      <c r="G13" s="32" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="32" t="s">
+        <v>348</v>
+      </c>
+      <c r="B14" s="32" t="s">
+        <v>349</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>350</v>
+      </c>
+      <c r="D14" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E14" s="32" t="s">
+        <v>351</v>
+      </c>
+      <c r="F14" s="32" t="s">
+        <v>352</v>
+      </c>
+      <c r="G14" s="32" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="32" t="s">
+        <v>348</v>
+      </c>
+      <c r="B15" s="32" t="s">
+        <v>354</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>324</v>
+      </c>
+      <c r="D15" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E15" s="32" t="s">
+        <v>355</v>
+      </c>
+      <c r="F15" s="32" t="s">
+        <v>322</v>
+      </c>
+      <c r="G15" s="32" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="32" t="s">
+        <v>348</v>
+      </c>
+      <c r="B16" s="32" t="s">
+        <v>354</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>252</v>
+      </c>
+      <c r="D16" s="32" t="s">
+        <v>328</v>
+      </c>
+      <c r="E16" s="32" t="s">
+        <v>357</v>
+      </c>
+      <c r="F16" s="32" t="s">
+        <v>345</v>
+      </c>
+      <c r="G16" s="32" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="32" t="s">
+        <v>358</v>
+      </c>
+      <c r="B17" s="32" t="s">
+        <v>359</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>360</v>
+      </c>
+      <c r="D17" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E17" s="32" t="s">
+        <v>361</v>
+      </c>
+      <c r="F17" s="32" t="s">
+        <v>352</v>
+      </c>
+      <c r="G17" s="32" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="32" t="s">
+        <v>358</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>363</v>
+      </c>
+      <c r="C18" s="32" t="s">
+        <v>275</v>
+      </c>
+      <c r="D18" s="32" t="s">
+        <v>328</v>
+      </c>
+      <c r="E18" s="32" t="s">
+        <v>364</v>
+      </c>
+      <c r="F18" s="32" t="s">
+        <v>352</v>
+      </c>
+      <c r="G18" s="32" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="32" t="s">
+        <v>365</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>366</v>
+      </c>
+      <c r="C19" s="32" t="s">
+        <v>367</v>
+      </c>
+      <c r="D19" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="E19" s="32" t="s">
+        <v>368</v>
+      </c>
+      <c r="F19" s="32" t="s">
+        <v>339</v>
+      </c>
+      <c r="G19" s="32" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="32" t="s">
+        <v>365</v>
+      </c>
+      <c r="B20" s="32" t="s">
+        <v>363</v>
+      </c>
+      <c r="C20" s="32" t="s">
+        <v>370</v>
+      </c>
+      <c r="D20" s="32" t="s">
+        <v>328</v>
+      </c>
+      <c r="E20" s="32" t="s">
+        <v>221</v>
+      </c>
+      <c r="F20" s="32" t="s">
+        <v>339</v>
+      </c>
+      <c r="G20" s="32" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="32"/>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+    </row>
+    <row r="22" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="33" t="s">
+        <v>371</v>
+      </c>
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+    </row>
+    <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="32" t="s">
+        <v>372</v>
+      </c>
+      <c r="B23" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+    </row>
+    <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="32" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="32" t="s">
+        <v>374</v>
+      </c>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="32" t="s">
+        <v>375</v>
+      </c>
+      <c r="B25" s="32" t="s">
+        <v>376</v>
+      </c>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+    </row>
+    <row r="26" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="32" t="s">
+        <v>377</v>
+      </c>
+      <c r="B26" s="32" t="s">
+        <v>378</v>
+      </c>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="32" t="s">
+        <v>379</v>
+      </c>
+      <c r="B27" s="32" t="s">
+        <v>380</v>
+      </c>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+    </row>
+    <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="32" t="s">
+        <v>381</v>
+      </c>
+      <c r="B28" s="32" t="s">
+        <v>382</v>
+      </c>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="32"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+    </row>
+    <row r="30" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="33" t="s">
+        <v>383</v>
+      </c>
+      <c r="B30" s="32" t="s">
+        <v>384</v>
+      </c>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>